<commit_message>
fix configuracion sp 17
</commit_message>
<xml_diff>
--- a/Guias Produccion/HU-64765.xlsx
+++ b/Guias Produccion/HU-64765.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Alliance\ScriptsEntidades\Guias Produccion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35DECB27-D2B2-44A5-B6FD-3A07D185C8B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B9B0329-24CC-4BDC-A5F1-0CF004E83A8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Guia de implementación" sheetId="1" r:id="rId1"/>
@@ -2247,89 +2247,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="12" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="50" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="51" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="52" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="53" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="54" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="59" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="63" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="60" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="64" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2433,6 +2352,90 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="50" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="51" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="52" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="53" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="54" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="59" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="63" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="60" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="64" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="71" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2504,9 +2507,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2609,11 +2609,11 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp113.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="[1]Hoja4!$A$1:$A$13" noThreeD="1" sel="0" val="0"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="1" val="0"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp114.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="1" val="0"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="2" val="0"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp115.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2633,7 +2633,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp119.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="[2]Hoja4!$A$1:$A$25" noThreeD="1" sel="0" val="0"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="2" val="0"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp12.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2641,30 +2641,10 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp120.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="[2]Hoja4!$A$1:$A$25" noThreeD="1" sel="0" val="0"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$17" noThreeD="1" sel="17" val="9"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp121.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="[2]Hoja4!$A$1:$A$25" noThreeD="1" sel="0" val="0"/>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp122.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="[2]Hoja4!$A$1:$A$25" noThreeD="1" sel="0" val="0"/>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp123.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="[2]Hoja4!$A$1:$A$25" noThreeD="1" sel="0" val="0"/>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp124.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="[2]Hoja4!$A$1:$A$25" noThreeD="1" sel="0" val="0"/>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp125.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$17" noThreeD="1" sel="17" val="9"/>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp126.xml><?xml version="1.0" encoding="utf-8"?>
 <formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$17" noThreeD="1" sel="17" val="9"/>
 </file>
 
@@ -9552,24 +9532,24 @@
         <xdr:from>
           <xdr:col>2</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>33</xdr:row>
+          <xdr:row>26</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>1409700</xdr:colOff>
-          <xdr:row>34</xdr:row>
-          <xdr:rowOff>38100</xdr:rowOff>
+          <xdr:row>26</xdr:row>
+          <xdr:rowOff>228600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="1208" name="Drop Down 184" hidden="1">
+            <xdr:cNvPr id="1223" name="Drop Down 199" hidden="1">
               <a:extLst>
                 <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1208"/>
+                  <a14:compatExt spid="_x0000_s1223"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000B8040000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000C7040000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -9610,24 +9590,24 @@
         <xdr:from>
           <xdr:col>2</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>26</xdr:row>
+          <xdr:row>27</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>1409700</xdr:colOff>
-          <xdr:row>26</xdr:row>
+          <xdr:row>27</xdr:row>
           <xdr:rowOff>228600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="1223" name="Drop Down 199" hidden="1">
+            <xdr:cNvPr id="1224" name="Drop Down 200" hidden="1">
               <a:extLst>
                 <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1223"/>
+                  <a14:compatExt spid="_x0000_s1224"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000C7040000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000C8040000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -9668,24 +9648,24 @@
         <xdr:from>
           <xdr:col>2</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>27</xdr:row>
+          <xdr:row>28</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>1409700</xdr:colOff>
-          <xdr:row>27</xdr:row>
+          <xdr:row>28</xdr:row>
           <xdr:rowOff>228600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="1224" name="Drop Down 200" hidden="1">
+            <xdr:cNvPr id="1226" name="Drop Down 202" hidden="1">
               <a:extLst>
                 <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1224"/>
+                  <a14:compatExt spid="_x0000_s1226"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000C8040000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000CA040000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -9726,24 +9706,24 @@
         <xdr:from>
           <xdr:col>2</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>28</xdr:row>
+          <xdr:row>29</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>1409700</xdr:colOff>
-          <xdr:row>28</xdr:row>
+          <xdr:row>29</xdr:row>
           <xdr:rowOff>228600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="1226" name="Drop Down 202" hidden="1">
+            <xdr:cNvPr id="1227" name="Drop Down 203" hidden="1">
               <a:extLst>
                 <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1226"/>
+                  <a14:compatExt spid="_x0000_s1227"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000CA040000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000CB040000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -9784,24 +9764,24 @@
         <xdr:from>
           <xdr:col>2</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>29</xdr:row>
+          <xdr:row>30</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>1409700</xdr:colOff>
-          <xdr:row>29</xdr:row>
+          <xdr:row>30</xdr:row>
           <xdr:rowOff>228600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="1227" name="Drop Down 203" hidden="1">
+            <xdr:cNvPr id="1228" name="Drop Down 204" hidden="1">
               <a:extLst>
                 <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1227"/>
+                  <a14:compatExt spid="_x0000_s1228"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000CB040000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000CC040000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -9842,24 +9822,24 @@
         <xdr:from>
           <xdr:col>2</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>30</xdr:row>
+          <xdr:row>31</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>1409700</xdr:colOff>
-          <xdr:row>30</xdr:row>
+          <xdr:row>31</xdr:row>
           <xdr:rowOff>228600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="1228" name="Drop Down 204" hidden="1">
+            <xdr:cNvPr id="1235" name="Drop Down 211" hidden="1">
               <a:extLst>
                 <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1228"/>
+                  <a14:compatExt spid="_x0000_s1235"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000CC040000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{97E19B0A-AA8C-956D-70DA-027CBC99120B}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -9900,296 +9880,6 @@
         <xdr:from>
           <xdr:col>2</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>27</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>1409700</xdr:colOff>
-          <xdr:row>27</xdr:row>
-          <xdr:rowOff>228600</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="1229" name="Drop Down 205" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1229"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000CD040000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:noFill/>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>28</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>1409700</xdr:colOff>
-          <xdr:row>28</xdr:row>
-          <xdr:rowOff>228600</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="1230" name="Drop Down 206" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1230"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000CE040000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:noFill/>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>29</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>1409700</xdr:colOff>
-          <xdr:row>29</xdr:row>
-          <xdr:rowOff>228600</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="1231" name="Drop Down 207" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1231"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000CF040000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:noFill/>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>30</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>1409700</xdr:colOff>
-          <xdr:row>30</xdr:row>
-          <xdr:rowOff>228600</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="1232" name="Drop Down 208" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1232"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000D0040000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:noFill/>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>31</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>1409700</xdr:colOff>
-          <xdr:row>31</xdr:row>
-          <xdr:rowOff>228600</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="1233" name="Drop Down 209" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1233"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000D1040000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:noFill/>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>2</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
           <xdr:row>32</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
@@ -10201,13 +9891,13 @@
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="1234" name="Drop Down 210" hidden="1">
+            <xdr:cNvPr id="1236" name="Drop Down 212" hidden="1">
               <a:extLst>
                 <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1234"/>
+                  <a14:compatExt spid="_x0000_s1236"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000D2040000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C43480FA-1092-7491-325B-B3820794AECC}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -10876,42 +10566,42 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:15" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="110" t="s">
+      <c r="A3" s="83" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="111"/>
-      <c r="C3" s="111"/>
-      <c r="D3" s="111"/>
-      <c r="E3" s="111"/>
-      <c r="F3" s="111"/>
-      <c r="G3" s="111"/>
-      <c r="H3" s="111"/>
-      <c r="I3" s="111"/>
-      <c r="J3" s="111"/>
-      <c r="K3" s="111"/>
-      <c r="L3" s="112"/>
-      <c r="N3" s="104" t="s">
+      <c r="B3" s="84"/>
+      <c r="C3" s="84"/>
+      <c r="D3" s="84"/>
+      <c r="E3" s="84"/>
+      <c r="F3" s="84"/>
+      <c r="G3" s="84"/>
+      <c r="H3" s="84"/>
+      <c r="I3" s="84"/>
+      <c r="J3" s="84"/>
+      <c r="K3" s="84"/>
+      <c r="L3" s="85"/>
+      <c r="N3" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="O3" s="105"/>
+      <c r="O3" s="78"/>
     </row>
     <row r="4" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="117" t="s">
+      <c r="B4" s="90" t="s">
         <v>110</v>
       </c>
-      <c r="C4" s="118"/>
-      <c r="D4" s="118"/>
-      <c r="E4" s="118"/>
-      <c r="F4" s="118"/>
-      <c r="G4" s="118"/>
-      <c r="H4" s="118"/>
-      <c r="I4" s="118"/>
-      <c r="J4" s="119"/>
-      <c r="K4" s="119"/>
-      <c r="L4" s="120"/>
+      <c r="C4" s="91"/>
+      <c r="D4" s="91"/>
+      <c r="E4" s="91"/>
+      <c r="F4" s="91"/>
+      <c r="G4" s="91"/>
+      <c r="H4" s="91"/>
+      <c r="I4" s="91"/>
+      <c r="J4" s="92"/>
+      <c r="K4" s="92"/>
+      <c r="L4" s="93"/>
       <c r="N4" s="20" t="s">
         <v>3</v>
       </c>
@@ -10921,19 +10611,19 @@
       <c r="A5" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="121" t="s">
+      <c r="B5" s="94" t="s">
         <v>109</v>
       </c>
-      <c r="C5" s="121"/>
-      <c r="D5" s="121"/>
-      <c r="E5" s="121"/>
-      <c r="F5" s="121"/>
-      <c r="G5" s="121"/>
-      <c r="H5" s="121"/>
-      <c r="I5" s="121"/>
-      <c r="J5" s="122"/>
-      <c r="K5" s="122"/>
-      <c r="L5" s="123"/>
+      <c r="C5" s="94"/>
+      <c r="D5" s="94"/>
+      <c r="E5" s="94"/>
+      <c r="F5" s="94"/>
+      <c r="G5" s="94"/>
+      <c r="H5" s="94"/>
+      <c r="I5" s="94"/>
+      <c r="J5" s="95"/>
+      <c r="K5" s="95"/>
+      <c r="L5" s="96"/>
       <c r="N5" s="14" t="s">
         <v>5</v>
       </c>
@@ -10943,19 +10633,19 @@
       <c r="A6" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="107">
+      <c r="B6" s="80">
         <v>46126</v>
       </c>
-      <c r="C6" s="108"/>
-      <c r="D6" s="108"/>
-      <c r="E6" s="108"/>
-      <c r="F6" s="108"/>
-      <c r="G6" s="108"/>
-      <c r="H6" s="108"/>
-      <c r="I6" s="108"/>
-      <c r="J6" s="108"/>
-      <c r="K6" s="108"/>
-      <c r="L6" s="109"/>
+      <c r="C6" s="81"/>
+      <c r="D6" s="81"/>
+      <c r="E6" s="81"/>
+      <c r="F6" s="81"/>
+      <c r="G6" s="81"/>
+      <c r="H6" s="81"/>
+      <c r="I6" s="81"/>
+      <c r="J6" s="81"/>
+      <c r="K6" s="81"/>
+      <c r="L6" s="82"/>
       <c r="N6" s="13"/>
       <c r="O6" s="13"/>
     </row>
@@ -10963,17 +10653,17 @@
       <c r="A7" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="124"/>
-      <c r="C7" s="125"/>
-      <c r="D7" s="125"/>
-      <c r="E7" s="125"/>
-      <c r="F7" s="125"/>
-      <c r="G7" s="125"/>
-      <c r="H7" s="125"/>
-      <c r="I7" s="125"/>
-      <c r="J7" s="126"/>
-      <c r="K7" s="126"/>
-      <c r="L7" s="127"/>
+      <c r="B7" s="97"/>
+      <c r="C7" s="98"/>
+      <c r="D7" s="98"/>
+      <c r="E7" s="98"/>
+      <c r="F7" s="98"/>
+      <c r="G7" s="98"/>
+      <c r="H7" s="98"/>
+      <c r="I7" s="98"/>
+      <c r="J7" s="99"/>
+      <c r="K7" s="99"/>
+      <c r="L7" s="100"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="10"/>
@@ -10990,20 +10680,20 @@
       <c r="L8" s="12"/>
     </row>
     <row r="9" spans="1:15" s="5" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="113" t="s">
+      <c r="A9" s="86" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="114"/>
-      <c r="C9" s="114"/>
-      <c r="D9" s="114"/>
-      <c r="E9" s="114"/>
-      <c r="F9" s="114"/>
-      <c r="G9" s="114"/>
-      <c r="H9" s="114"/>
-      <c r="I9" s="114"/>
-      <c r="J9" s="115"/>
-      <c r="K9" s="115"/>
-      <c r="L9" s="116"/>
+      <c r="B9" s="87"/>
+      <c r="C9" s="87"/>
+      <c r="D9" s="87"/>
+      <c r="E9" s="87"/>
+      <c r="F9" s="87"/>
+      <c r="G9" s="87"/>
+      <c r="H9" s="87"/>
+      <c r="I9" s="87"/>
+      <c r="J9" s="88"/>
+      <c r="K9" s="88"/>
+      <c r="L9" s="89"/>
     </row>
     <row r="10" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
@@ -11095,63 +10785,63 @@
       <c r="A14" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="106"/>
-      <c r="C14" s="102"/>
-      <c r="D14" s="102"/>
-      <c r="E14" s="102"/>
-      <c r="F14" s="102"/>
-      <c r="G14" s="102"/>
-      <c r="H14" s="102"/>
-      <c r="I14" s="102"/>
-      <c r="J14" s="102"/>
-      <c r="K14" s="102"/>
-      <c r="L14" s="103"/>
+      <c r="B14" s="79"/>
+      <c r="C14" s="75"/>
+      <c r="D14" s="75"/>
+      <c r="E14" s="75"/>
+      <c r="F14" s="75"/>
+      <c r="G14" s="75"/>
+      <c r="H14" s="75"/>
+      <c r="I14" s="75"/>
+      <c r="J14" s="75"/>
+      <c r="K14" s="75"/>
+      <c r="L14" s="76"/>
     </row>
     <row r="15" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="101"/>
-      <c r="C15" s="102"/>
-      <c r="D15" s="102"/>
-      <c r="E15" s="102"/>
-      <c r="F15" s="102"/>
-      <c r="G15" s="102"/>
-      <c r="H15" s="102"/>
-      <c r="I15" s="102"/>
-      <c r="J15" s="102"/>
-      <c r="K15" s="102"/>
-      <c r="L15" s="103"/>
+      <c r="B15" s="74"/>
+      <c r="C15" s="75"/>
+      <c r="D15" s="75"/>
+      <c r="E15" s="75"/>
+      <c r="F15" s="75"/>
+      <c r="G15" s="75"/>
+      <c r="H15" s="75"/>
+      <c r="I15" s="75"/>
+      <c r="J15" s="75"/>
+      <c r="K15" s="75"/>
+      <c r="L15" s="76"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A16" s="94"/>
-      <c r="B16" s="95"/>
-      <c r="C16" s="95"/>
-      <c r="D16" s="95"/>
-      <c r="E16" s="95"/>
-      <c r="F16" s="95"/>
-      <c r="G16" s="95"/>
-      <c r="H16" s="95"/>
-      <c r="I16" s="95"/>
-      <c r="J16" s="95"/>
-      <c r="K16" s="95"/>
-      <c r="L16" s="96"/>
+      <c r="A16" s="67"/>
+      <c r="B16" s="68"/>
+      <c r="C16" s="68"/>
+      <c r="D16" s="68"/>
+      <c r="E16" s="68"/>
+      <c r="F16" s="68"/>
+      <c r="G16" s="68"/>
+      <c r="H16" s="68"/>
+      <c r="I16" s="68"/>
+      <c r="J16" s="68"/>
+      <c r="K16" s="68"/>
+      <c r="L16" s="69"/>
     </row>
     <row r="17" spans="1:13" s="5" customFormat="1" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="97" t="s">
+      <c r="A17" s="70" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="98"/>
-      <c r="C17" s="98"/>
-      <c r="D17" s="98"/>
-      <c r="E17" s="98"/>
-      <c r="F17" s="98"/>
-      <c r="G17" s="98"/>
-      <c r="H17" s="98"/>
-      <c r="I17" s="98"/>
-      <c r="J17" s="99"/>
-      <c r="K17" s="99"/>
-      <c r="L17" s="100"/>
+      <c r="B17" s="71"/>
+      <c r="C17" s="71"/>
+      <c r="D17" s="71"/>
+      <c r="E17" s="71"/>
+      <c r="F17" s="71"/>
+      <c r="G17" s="71"/>
+      <c r="H17" s="71"/>
+      <c r="I17" s="71"/>
+      <c r="J17" s="72"/>
+      <c r="K17" s="72"/>
+      <c r="L17" s="73"/>
     </row>
     <row r="18" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="47" t="s">
@@ -11163,17 +10853,17 @@
       <c r="C18" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="D18" s="72" t="s">
+      <c r="D18" s="107" t="s">
         <v>30</v>
       </c>
-      <c r="E18" s="74"/>
-      <c r="F18" s="74"/>
-      <c r="G18" s="74"/>
-      <c r="H18" s="74"/>
-      <c r="I18" s="74"/>
-      <c r="J18" s="75"/>
-      <c r="K18" s="75"/>
-      <c r="L18" s="76"/>
+      <c r="E18" s="109"/>
+      <c r="F18" s="109"/>
+      <c r="G18" s="109"/>
+      <c r="H18" s="109"/>
+      <c r="I18" s="109"/>
+      <c r="J18" s="110"/>
+      <c r="K18" s="110"/>
+      <c r="L18" s="111"/>
     </row>
     <row r="19" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
@@ -11183,15 +10873,15 @@
       <c r="C19" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="D19" s="73"/>
-      <c r="E19" s="77"/>
-      <c r="F19" s="77"/>
-      <c r="G19" s="77"/>
-      <c r="H19" s="77"/>
-      <c r="I19" s="77"/>
-      <c r="J19" s="78"/>
-      <c r="K19" s="78"/>
-      <c r="L19" s="79"/>
+      <c r="D19" s="108"/>
+      <c r="E19" s="112"/>
+      <c r="F19" s="112"/>
+      <c r="G19" s="112"/>
+      <c r="H19" s="112"/>
+      <c r="I19" s="112"/>
+      <c r="J19" s="113"/>
+      <c r="K19" s="113"/>
+      <c r="L19" s="114"/>
     </row>
     <row r="20" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
@@ -11201,15 +10891,15 @@
         <v>32</v>
       </c>
       <c r="C20" s="32"/>
-      <c r="D20" s="73"/>
-      <c r="E20" s="77"/>
-      <c r="F20" s="77"/>
-      <c r="G20" s="77"/>
-      <c r="H20" s="77"/>
-      <c r="I20" s="77"/>
-      <c r="J20" s="78"/>
-      <c r="K20" s="78"/>
-      <c r="L20" s="79"/>
+      <c r="D20" s="108"/>
+      <c r="E20" s="112"/>
+      <c r="F20" s="112"/>
+      <c r="G20" s="112"/>
+      <c r="H20" s="112"/>
+      <c r="I20" s="112"/>
+      <c r="J20" s="113"/>
+      <c r="K20" s="113"/>
+      <c r="L20" s="114"/>
     </row>
     <row r="21" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
@@ -11219,20 +10909,20 @@
       <c r="C21" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="D21" s="88" t="s">
+      <c r="D21" s="123" t="s">
         <v>26</v>
       </c>
-      <c r="E21" s="90" t="s">
+      <c r="E21" s="125" t="s">
         <v>106</v>
       </c>
-      <c r="F21" s="91"/>
-      <c r="G21" s="91"/>
-      <c r="H21" s="91"/>
-      <c r="I21" s="91"/>
-      <c r="J21" s="91"/>
-      <c r="K21" s="91"/>
-      <c r="L21" s="91"/>
-      <c r="M21" s="91"/>
+      <c r="F21" s="126"/>
+      <c r="G21" s="126"/>
+      <c r="H21" s="126"/>
+      <c r="I21" s="126"/>
+      <c r="J21" s="126"/>
+      <c r="K21" s="126"/>
+      <c r="L21" s="126"/>
+      <c r="M21" s="126"/>
     </row>
     <row r="22" spans="1:13" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="7" t="s">
@@ -11242,46 +10932,46 @@
       <c r="C22" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="D22" s="89"/>
-      <c r="E22" s="92"/>
-      <c r="F22" s="93"/>
-      <c r="G22" s="93"/>
-      <c r="H22" s="93"/>
-      <c r="I22" s="93"/>
-      <c r="J22" s="93"/>
-      <c r="K22" s="93"/>
-      <c r="L22" s="93"/>
-      <c r="M22" s="93"/>
+      <c r="D22" s="124"/>
+      <c r="E22" s="127"/>
+      <c r="F22" s="128"/>
+      <c r="G22" s="128"/>
+      <c r="H22" s="128"/>
+      <c r="I22" s="128"/>
+      <c r="J22" s="128"/>
+      <c r="K22" s="128"/>
+      <c r="L22" s="128"/>
+      <c r="M22" s="128"/>
     </row>
     <row r="23" spans="1:13" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="81"/>
-      <c r="B23" s="82"/>
-      <c r="C23" s="82"/>
-      <c r="D23" s="83"/>
-      <c r="E23" s="83"/>
-      <c r="F23" s="83"/>
-      <c r="G23" s="83"/>
-      <c r="H23" s="83"/>
-      <c r="I23" s="83"/>
-      <c r="J23" s="83"/>
-      <c r="K23" s="83"/>
-      <c r="L23" s="84"/>
+      <c r="A23" s="116"/>
+      <c r="B23" s="117"/>
+      <c r="C23" s="117"/>
+      <c r="D23" s="118"/>
+      <c r="E23" s="118"/>
+      <c r="F23" s="118"/>
+      <c r="G23" s="118"/>
+      <c r="H23" s="118"/>
+      <c r="I23" s="118"/>
+      <c r="J23" s="118"/>
+      <c r="K23" s="118"/>
+      <c r="L23" s="119"/>
     </row>
     <row r="24" spans="1:13" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="85" t="s">
+      <c r="A24" s="120" t="s">
         <v>36</v>
       </c>
-      <c r="B24" s="86"/>
-      <c r="C24" s="86"/>
-      <c r="D24" s="86"/>
-      <c r="E24" s="86"/>
-      <c r="F24" s="86"/>
-      <c r="G24" s="86"/>
-      <c r="H24" s="86"/>
-      <c r="I24" s="86"/>
-      <c r="J24" s="86"/>
-      <c r="K24" s="86"/>
-      <c r="L24" s="87"/>
+      <c r="B24" s="121"/>
+      <c r="C24" s="121"/>
+      <c r="D24" s="121"/>
+      <c r="E24" s="121"/>
+      <c r="F24" s="121"/>
+      <c r="G24" s="121"/>
+      <c r="H24" s="121"/>
+      <c r="I24" s="121"/>
+      <c r="J24" s="121"/>
+      <c r="K24" s="121"/>
+      <c r="L24" s="122"/>
     </row>
     <row r="25" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="15" t="s">
@@ -11293,17 +10983,17 @@
       <c r="C25" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="D25" s="80" t="s">
+      <c r="D25" s="115" t="s">
         <v>40</v>
       </c>
-      <c r="E25" s="80"/>
-      <c r="F25" s="80"/>
-      <c r="G25" s="80"/>
-      <c r="H25" s="80"/>
-      <c r="I25" s="80"/>
-      <c r="J25" s="80"/>
-      <c r="K25" s="80"/>
-      <c r="L25" s="80"/>
+      <c r="E25" s="115"/>
+      <c r="F25" s="115"/>
+      <c r="G25" s="115"/>
+      <c r="H25" s="115"/>
+      <c r="I25" s="115"/>
+      <c r="J25" s="115"/>
+      <c r="K25" s="115"/>
+      <c r="L25" s="115"/>
     </row>
     <row r="26" spans="1:13" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="64">
@@ -11313,17 +11003,17 @@
         <v>112</v>
       </c>
       <c r="C26" s="25"/>
-      <c r="D26" s="66" t="s">
+      <c r="D26" s="101" t="s">
         <v>120</v>
       </c>
-      <c r="E26" s="67"/>
-      <c r="F26" s="67"/>
-      <c r="G26" s="67"/>
-      <c r="H26" s="67"/>
-      <c r="I26" s="67"/>
-      <c r="J26" s="67"/>
-      <c r="K26" s="67"/>
-      <c r="L26" s="68"/>
+      <c r="E26" s="102"/>
+      <c r="F26" s="102"/>
+      <c r="G26" s="102"/>
+      <c r="H26" s="102"/>
+      <c r="I26" s="102"/>
+      <c r="J26" s="102"/>
+      <c r="K26" s="102"/>
+      <c r="L26" s="103"/>
     </row>
     <row r="27" spans="1:13" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="64">
@@ -11333,15 +11023,15 @@
         <v>113</v>
       </c>
       <c r="C27" s="25"/>
-      <c r="D27" s="69"/>
-      <c r="E27" s="70"/>
-      <c r="F27" s="70"/>
-      <c r="G27" s="70"/>
-      <c r="H27" s="70"/>
-      <c r="I27" s="70"/>
-      <c r="J27" s="70"/>
-      <c r="K27" s="70"/>
-      <c r="L27" s="71"/>
+      <c r="D27" s="104"/>
+      <c r="E27" s="105"/>
+      <c r="F27" s="105"/>
+      <c r="G27" s="105"/>
+      <c r="H27" s="105"/>
+      <c r="I27" s="105"/>
+      <c r="J27" s="105"/>
+      <c r="K27" s="105"/>
+      <c r="L27" s="106"/>
     </row>
     <row r="28" spans="1:13" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="24">
@@ -11351,15 +11041,15 @@
         <v>114</v>
       </c>
       <c r="C28" s="25"/>
-      <c r="D28" s="69"/>
-      <c r="E28" s="70"/>
-      <c r="F28" s="70"/>
-      <c r="G28" s="70"/>
-      <c r="H28" s="70"/>
-      <c r="I28" s="70"/>
-      <c r="J28" s="70"/>
-      <c r="K28" s="70"/>
-      <c r="L28" s="71"/>
+      <c r="D28" s="104"/>
+      <c r="E28" s="105"/>
+      <c r="F28" s="105"/>
+      <c r="G28" s="105"/>
+      <c r="H28" s="105"/>
+      <c r="I28" s="105"/>
+      <c r="J28" s="105"/>
+      <c r="K28" s="105"/>
+      <c r="L28" s="106"/>
     </row>
     <row r="29" spans="1:13" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="24">
@@ -11369,15 +11059,15 @@
         <v>115</v>
       </c>
       <c r="C29" s="25"/>
-      <c r="D29" s="69"/>
-      <c r="E29" s="70"/>
-      <c r="F29" s="70"/>
-      <c r="G29" s="70"/>
-      <c r="H29" s="70"/>
-      <c r="I29" s="70"/>
-      <c r="J29" s="70"/>
-      <c r="K29" s="70"/>
-      <c r="L29" s="71"/>
+      <c r="D29" s="104"/>
+      <c r="E29" s="105"/>
+      <c r="F29" s="105"/>
+      <c r="G29" s="105"/>
+      <c r="H29" s="105"/>
+      <c r="I29" s="105"/>
+      <c r="J29" s="105"/>
+      <c r="K29" s="105"/>
+      <c r="L29" s="106"/>
     </row>
     <row r="30" spans="1:13" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="24">
@@ -11387,15 +11077,15 @@
         <v>116</v>
       </c>
       <c r="C30" s="25"/>
-      <c r="D30" s="69"/>
-      <c r="E30" s="70"/>
-      <c r="F30" s="70"/>
-      <c r="G30" s="70"/>
-      <c r="H30" s="70"/>
-      <c r="I30" s="70"/>
-      <c r="J30" s="70"/>
-      <c r="K30" s="70"/>
-      <c r="L30" s="71"/>
+      <c r="D30" s="104"/>
+      <c r="E30" s="105"/>
+      <c r="F30" s="105"/>
+      <c r="G30" s="105"/>
+      <c r="H30" s="105"/>
+      <c r="I30" s="105"/>
+      <c r="J30" s="105"/>
+      <c r="K30" s="105"/>
+      <c r="L30" s="106"/>
     </row>
     <row r="31" spans="1:13" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="24">
@@ -11405,15 +11095,15 @@
         <v>117</v>
       </c>
       <c r="C31" s="25"/>
-      <c r="D31" s="69"/>
-      <c r="E31" s="70"/>
-      <c r="F31" s="70"/>
-      <c r="G31" s="70"/>
-      <c r="H31" s="70"/>
-      <c r="I31" s="70"/>
-      <c r="J31" s="70"/>
-      <c r="K31" s="70"/>
-      <c r="L31" s="71"/>
+      <c r="D31" s="104"/>
+      <c r="E31" s="105"/>
+      <c r="F31" s="105"/>
+      <c r="G31" s="105"/>
+      <c r="H31" s="105"/>
+      <c r="I31" s="105"/>
+      <c r="J31" s="105"/>
+      <c r="K31" s="105"/>
+      <c r="L31" s="106"/>
     </row>
     <row r="32" spans="1:13" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="24">
@@ -11423,15 +11113,15 @@
         <v>118</v>
       </c>
       <c r="C32" s="25"/>
-      <c r="D32" s="69"/>
-      <c r="E32" s="70"/>
-      <c r="F32" s="70"/>
-      <c r="G32" s="70"/>
-      <c r="H32" s="70"/>
-      <c r="I32" s="70"/>
-      <c r="J32" s="70"/>
-      <c r="K32" s="70"/>
-      <c r="L32" s="71"/>
+      <c r="D32" s="104"/>
+      <c r="E32" s="105"/>
+      <c r="F32" s="105"/>
+      <c r="G32" s="105"/>
+      <c r="H32" s="105"/>
+      <c r="I32" s="105"/>
+      <c r="J32" s="105"/>
+      <c r="K32" s="105"/>
+      <c r="L32" s="106"/>
     </row>
     <row r="33" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="24">
@@ -11441,18 +11131,26 @@
         <v>119</v>
       </c>
       <c r="C33" s="25"/>
-      <c r="D33" s="69"/>
-      <c r="E33" s="70"/>
-      <c r="F33" s="70"/>
-      <c r="G33" s="70"/>
-      <c r="H33" s="70"/>
-      <c r="I33" s="70"/>
-      <c r="J33" s="70"/>
-      <c r="K33" s="70"/>
-      <c r="L33" s="71"/>
+      <c r="D33" s="104"/>
+      <c r="E33" s="105"/>
+      <c r="F33" s="105"/>
+      <c r="G33" s="105"/>
+      <c r="H33" s="105"/>
+      <c r="I33" s="105"/>
+      <c r="J33" s="105"/>
+      <c r="K33" s="105"/>
+      <c r="L33" s="106"/>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="D26:L33"/>
+    <mergeCell ref="D18:D20"/>
+    <mergeCell ref="E18:L20"/>
+    <mergeCell ref="D25:L25"/>
+    <mergeCell ref="A23:L23"/>
+    <mergeCell ref="A24:L24"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="E21:M22"/>
     <mergeCell ref="A16:L16"/>
     <mergeCell ref="A17:L17"/>
     <mergeCell ref="B15:L15"/>
@@ -11464,14 +11162,6 @@
     <mergeCell ref="B4:L4"/>
     <mergeCell ref="B5:L5"/>
     <mergeCell ref="B7:L7"/>
-    <mergeCell ref="D26:L33"/>
-    <mergeCell ref="D18:D20"/>
-    <mergeCell ref="E18:L20"/>
-    <mergeCell ref="D25:L25"/>
-    <mergeCell ref="A23:L23"/>
-    <mergeCell ref="A24:L24"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="E21:M22"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D26" r:id="rId1" xr:uid="{066995C9-04C2-4C67-9A74-29047F42F145}"/>
@@ -13949,29 +13639,7 @@
         </mc:AlternateContent>
         <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
           <mc:Choice Requires="x14">
-            <control shapeId="1208" r:id="rId117" name="Drop Down 184">
-              <controlPr defaultSize="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>0</xdr:colOff>
-                    <xdr:row>33</xdr:row>
-                    <xdr:rowOff>0</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>1409700</xdr:colOff>
-                    <xdr:row>34</xdr:row>
-                    <xdr:rowOff>38100</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="1223" r:id="rId118" name="Drop Down 199">
+            <control shapeId="1223" r:id="rId117" name="Drop Down 199">
               <controlPr defaultSize="0" autoLine="0" autoPict="0">
                 <anchor moveWithCells="1">
                   <from>
@@ -13993,7 +13661,7 @@
         </mc:AlternateContent>
         <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
           <mc:Choice Requires="x14">
-            <control shapeId="1224" r:id="rId119" name="Drop Down 200">
+            <control shapeId="1224" r:id="rId118" name="Drop Down 200">
               <controlPr defaultSize="0" autoLine="0" autoPict="0">
                 <anchor moveWithCells="1">
                   <from>
@@ -14015,7 +13683,7 @@
         </mc:AlternateContent>
         <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
           <mc:Choice Requires="x14">
-            <control shapeId="1226" r:id="rId120" name="Drop Down 202">
+            <control shapeId="1226" r:id="rId119" name="Drop Down 202">
               <controlPr defaultSize="0" autoLine="0" autoPict="0">
                 <anchor moveWithCells="1">
                   <from>
@@ -14037,7 +13705,7 @@
         </mc:AlternateContent>
         <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
           <mc:Choice Requires="x14">
-            <control shapeId="1227" r:id="rId121" name="Drop Down 203">
+            <control shapeId="1227" r:id="rId120" name="Drop Down 203">
               <controlPr defaultSize="0" autoLine="0" autoPict="0">
                 <anchor moveWithCells="1">
                   <from>
@@ -14059,7 +13727,7 @@
         </mc:AlternateContent>
         <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
           <mc:Choice Requires="x14">
-            <control shapeId="1228" r:id="rId122" name="Drop Down 204">
+            <control shapeId="1228" r:id="rId121" name="Drop Down 204">
               <controlPr defaultSize="0" autoLine="0" autoPict="0">
                 <anchor moveWithCells="1">
                   <from>
@@ -14081,95 +13749,7 @@
         </mc:AlternateContent>
         <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
           <mc:Choice Requires="x14">
-            <control shapeId="1229" r:id="rId123" name="Drop Down 205">
-              <controlPr defaultSize="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>0</xdr:colOff>
-                    <xdr:row>27</xdr:row>
-                    <xdr:rowOff>0</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>1409700</xdr:colOff>
-                    <xdr:row>27</xdr:row>
-                    <xdr:rowOff>228600</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="1230" r:id="rId124" name="Drop Down 206">
-              <controlPr defaultSize="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>0</xdr:colOff>
-                    <xdr:row>28</xdr:row>
-                    <xdr:rowOff>0</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>1409700</xdr:colOff>
-                    <xdr:row>28</xdr:row>
-                    <xdr:rowOff>228600</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="1231" r:id="rId125" name="Drop Down 207">
-              <controlPr defaultSize="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>0</xdr:colOff>
-                    <xdr:row>29</xdr:row>
-                    <xdr:rowOff>0</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>1409700</xdr:colOff>
-                    <xdr:row>29</xdr:row>
-                    <xdr:rowOff>228600</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="1232" r:id="rId126" name="Drop Down 208">
-              <controlPr defaultSize="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>0</xdr:colOff>
-                    <xdr:row>30</xdr:row>
-                    <xdr:rowOff>0</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>2</xdr:col>
-                    <xdr:colOff>1409700</xdr:colOff>
-                    <xdr:row>30</xdr:row>
-                    <xdr:rowOff>228600</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="1233" r:id="rId127" name="Drop Down 209">
+            <control shapeId="1235" r:id="rId122" name="Drop Down 211">
               <controlPr defaultSize="0" autoLine="0" autoPict="0">
                 <anchor moveWithCells="1">
                   <from>
@@ -14191,7 +13771,7 @@
         </mc:AlternateContent>
         <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
           <mc:Choice Requires="x14">
-            <control shapeId="1234" r:id="rId128" name="Drop Down 210">
+            <control shapeId="1236" r:id="rId123" name="Drop Down 212">
               <controlPr defaultSize="0" autoLine="0" autoPict="0">
                 <anchor moveWithCells="1">
                   <from>
@@ -14236,50 +13816,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="23.4" x14ac:dyDescent="0.3">
-      <c r="A1" s="137" t="s">
+      <c r="A1" s="138" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="138"/>
-      <c r="C1" s="138"/>
-      <c r="D1" s="138"/>
-      <c r="E1" s="138"/>
-      <c r="F1" s="138"/>
-      <c r="G1" s="138"/>
-      <c r="H1" s="138"/>
-      <c r="I1" s="138"/>
-      <c r="J1" s="138"/>
-      <c r="K1" s="138"/>
-      <c r="L1" s="139"/>
+      <c r="B1" s="139"/>
+      <c r="C1" s="139"/>
+      <c r="D1" s="139"/>
+      <c r="E1" s="139"/>
+      <c r="F1" s="139"/>
+      <c r="G1" s="139"/>
+      <c r="H1" s="139"/>
+      <c r="I1" s="139"/>
+      <c r="J1" s="139"/>
+      <c r="K1" s="139"/>
+      <c r="L1" s="140"/>
     </row>
     <row r="2" spans="1:12" ht="24" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="140" t="s">
+      <c r="A2" s="141" t="s">
         <v>42</v>
       </c>
-      <c r="B2" s="141"/>
-      <c r="C2" s="141"/>
-      <c r="D2" s="141"/>
-      <c r="E2" s="141"/>
-      <c r="F2" s="141"/>
-      <c r="G2" s="141"/>
-      <c r="H2" s="141"/>
-      <c r="I2" s="141"/>
-      <c r="J2" s="141"/>
-      <c r="K2" s="141"/>
-      <c r="L2" s="142"/>
+      <c r="B2" s="142"/>
+      <c r="C2" s="142"/>
+      <c r="D2" s="142"/>
+      <c r="E2" s="142"/>
+      <c r="F2" s="142"/>
+      <c r="G2" s="142"/>
+      <c r="H2" s="142"/>
+      <c r="I2" s="142"/>
+      <c r="J2" s="142"/>
+      <c r="K2" s="142"/>
+      <c r="L2" s="143"/>
     </row>
     <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="143"/>
-      <c r="B3" s="144"/>
-      <c r="C3" s="144"/>
-      <c r="D3" s="144"/>
-      <c r="E3" s="144"/>
-      <c r="F3" s="144"/>
-      <c r="G3" s="144"/>
-      <c r="H3" s="144"/>
-      <c r="I3" s="144"/>
-      <c r="J3" s="144"/>
-      <c r="K3" s="144"/>
-      <c r="L3" s="145"/>
+      <c r="A3" s="144"/>
+      <c r="B3" s="145"/>
+      <c r="C3" s="145"/>
+      <c r="D3" s="145"/>
+      <c r="E3" s="145"/>
+      <c r="F3" s="145"/>
+      <c r="G3" s="145"/>
+      <c r="H3" s="145"/>
+      <c r="I3" s="145"/>
+      <c r="J3" s="145"/>
+      <c r="K3" s="145"/>
+      <c r="L3" s="146"/>
     </row>
     <row r="4" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
@@ -14369,65 +13949,65 @@
       <c r="A8" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="148"/>
-      <c r="C8" s="149"/>
-      <c r="D8" s="149"/>
-      <c r="E8" s="149"/>
-      <c r="F8" s="149"/>
-      <c r="G8" s="149"/>
-      <c r="H8" s="149"/>
-      <c r="I8" s="149"/>
-      <c r="J8" s="149"/>
-      <c r="K8" s="149"/>
-      <c r="L8" s="150"/>
+      <c r="B8" s="149"/>
+      <c r="C8" s="150"/>
+      <c r="D8" s="150"/>
+      <c r="E8" s="150"/>
+      <c r="F8" s="150"/>
+      <c r="G8" s="150"/>
+      <c r="H8" s="150"/>
+      <c r="I8" s="150"/>
+      <c r="J8" s="150"/>
+      <c r="K8" s="150"/>
+      <c r="L8" s="151"/>
     </row>
     <row r="9" spans="1:12" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="151"/>
-      <c r="C9" s="149"/>
-      <c r="D9" s="149"/>
-      <c r="E9" s="149"/>
-      <c r="F9" s="149"/>
-      <c r="G9" s="149"/>
-      <c r="H9" s="149"/>
-      <c r="I9" s="149"/>
-      <c r="J9" s="149"/>
-      <c r="K9" s="149"/>
-      <c r="L9" s="150"/>
+      <c r="B9" s="152"/>
+      <c r="C9" s="150"/>
+      <c r="D9" s="150"/>
+      <c r="E9" s="150"/>
+      <c r="F9" s="150"/>
+      <c r="G9" s="150"/>
+      <c r="H9" s="150"/>
+      <c r="I9" s="150"/>
+      <c r="J9" s="150"/>
+      <c r="K9" s="150"/>
+      <c r="L9" s="151"/>
     </row>
     <row r="10" spans="1:12" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="146" t="s">
+      <c r="A10" s="147" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="147"/>
-      <c r="C10" s="147"/>
-      <c r="D10" s="147"/>
-      <c r="E10" s="147"/>
-      <c r="F10" s="147"/>
-      <c r="G10" s="147"/>
-      <c r="H10" s="147"/>
-      <c r="I10" s="147"/>
-      <c r="J10" s="147"/>
-      <c r="K10" s="147"/>
-      <c r="L10" s="147"/>
+      <c r="B10" s="148"/>
+      <c r="C10" s="148"/>
+      <c r="D10" s="148"/>
+      <c r="E10" s="148"/>
+      <c r="F10" s="148"/>
+      <c r="G10" s="148"/>
+      <c r="H10" s="148"/>
+      <c r="I10" s="148"/>
+      <c r="J10" s="148"/>
+      <c r="K10" s="148"/>
+      <c r="L10" s="148"/>
     </row>
     <row r="11" spans="1:12" ht="24" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="128" t="s">
+      <c r="A11" s="129" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="129"/>
-      <c r="C11" s="129"/>
-      <c r="D11" s="129"/>
-      <c r="E11" s="129"/>
-      <c r="F11" s="129"/>
-      <c r="G11" s="129"/>
-      <c r="H11" s="129"/>
-      <c r="I11" s="129"/>
-      <c r="J11" s="129"/>
-      <c r="K11" s="129"/>
-      <c r="L11" s="130"/>
+      <c r="B11" s="130"/>
+      <c r="C11" s="130"/>
+      <c r="D11" s="130"/>
+      <c r="E11" s="130"/>
+      <c r="F11" s="130"/>
+      <c r="G11" s="130"/>
+      <c r="H11" s="130"/>
+      <c r="I11" s="130"/>
+      <c r="J11" s="130"/>
+      <c r="K11" s="130"/>
+      <c r="L11" s="131"/>
     </row>
     <row r="12" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="15" t="s">
@@ -14439,101 +14019,101 @@
       <c r="C12" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="80" t="s">
+      <c r="D12" s="115" t="s">
         <v>40</v>
       </c>
-      <c r="E12" s="80"/>
-      <c r="F12" s="80"/>
-      <c r="G12" s="80"/>
-      <c r="H12" s="80"/>
-      <c r="I12" s="80"/>
-      <c r="J12" s="80"/>
-      <c r="K12" s="80"/>
-      <c r="L12" s="80"/>
+      <c r="E12" s="115"/>
+      <c r="F12" s="115"/>
+      <c r="G12" s="115"/>
+      <c r="H12" s="115"/>
+      <c r="I12" s="115"/>
+      <c r="J12" s="115"/>
+      <c r="K12" s="115"/>
+      <c r="L12" s="115"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="36"/>
       <c r="B13" s="37"/>
       <c r="C13" s="37"/>
-      <c r="D13" s="131"/>
-      <c r="E13" s="132"/>
-      <c r="F13" s="132"/>
-      <c r="G13" s="132"/>
-      <c r="H13" s="132"/>
-      <c r="I13" s="132"/>
-      <c r="J13" s="132"/>
-      <c r="K13" s="132"/>
-      <c r="L13" s="133"/>
+      <c r="D13" s="132"/>
+      <c r="E13" s="133"/>
+      <c r="F13" s="133"/>
+      <c r="G13" s="133"/>
+      <c r="H13" s="133"/>
+      <c r="I13" s="133"/>
+      <c r="J13" s="133"/>
+      <c r="K13" s="133"/>
+      <c r="L13" s="134"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="36"/>
       <c r="B14" s="37"/>
       <c r="C14" s="37"/>
-      <c r="D14" s="134"/>
-      <c r="E14" s="135"/>
-      <c r="F14" s="135"/>
-      <c r="G14" s="135"/>
-      <c r="H14" s="135"/>
-      <c r="I14" s="135"/>
-      <c r="J14" s="135"/>
-      <c r="K14" s="135"/>
-      <c r="L14" s="136"/>
+      <c r="D14" s="135"/>
+      <c r="E14" s="136"/>
+      <c r="F14" s="136"/>
+      <c r="G14" s="136"/>
+      <c r="H14" s="136"/>
+      <c r="I14" s="136"/>
+      <c r="J14" s="136"/>
+      <c r="K14" s="136"/>
+      <c r="L14" s="137"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="36"/>
       <c r="B15" s="37"/>
       <c r="C15" s="37"/>
-      <c r="D15" s="134"/>
-      <c r="E15" s="135"/>
-      <c r="F15" s="135"/>
-      <c r="G15" s="135"/>
-      <c r="H15" s="135"/>
-      <c r="I15" s="135"/>
-      <c r="J15" s="135"/>
-      <c r="K15" s="135"/>
-      <c r="L15" s="136"/>
+      <c r="D15" s="135"/>
+      <c r="E15" s="136"/>
+      <c r="F15" s="136"/>
+      <c r="G15" s="136"/>
+      <c r="H15" s="136"/>
+      <c r="I15" s="136"/>
+      <c r="J15" s="136"/>
+      <c r="K15" s="136"/>
+      <c r="L15" s="137"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="36"/>
       <c r="B16" s="37"/>
       <c r="C16" s="37"/>
-      <c r="D16" s="134"/>
-      <c r="E16" s="135"/>
-      <c r="F16" s="135"/>
-      <c r="G16" s="135"/>
-      <c r="H16" s="135"/>
-      <c r="I16" s="135"/>
-      <c r="J16" s="135"/>
-      <c r="K16" s="135"/>
-      <c r="L16" s="136"/>
+      <c r="D16" s="135"/>
+      <c r="E16" s="136"/>
+      <c r="F16" s="136"/>
+      <c r="G16" s="136"/>
+      <c r="H16" s="136"/>
+      <c r="I16" s="136"/>
+      <c r="J16" s="136"/>
+      <c r="K16" s="136"/>
+      <c r="L16" s="137"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="36"/>
       <c r="B17" s="37"/>
       <c r="C17" s="37"/>
-      <c r="D17" s="134"/>
-      <c r="E17" s="135"/>
-      <c r="F17" s="135"/>
-      <c r="G17" s="135"/>
-      <c r="H17" s="135"/>
-      <c r="I17" s="135"/>
-      <c r="J17" s="135"/>
-      <c r="K17" s="135"/>
-      <c r="L17" s="136"/>
+      <c r="D17" s="135"/>
+      <c r="E17" s="136"/>
+      <c r="F17" s="136"/>
+      <c r="G17" s="136"/>
+      <c r="H17" s="136"/>
+      <c r="I17" s="136"/>
+      <c r="J17" s="136"/>
+      <c r="K17" s="136"/>
+      <c r="L17" s="137"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="36"/>
       <c r="B18" s="37"/>
       <c r="C18" s="37"/>
-      <c r="D18" s="134"/>
-      <c r="E18" s="135"/>
-      <c r="F18" s="135"/>
-      <c r="G18" s="135"/>
-      <c r="H18" s="135"/>
-      <c r="I18" s="135"/>
-      <c r="J18" s="135"/>
-      <c r="K18" s="135"/>
-      <c r="L18" s="136"/>
+      <c r="D18" s="135"/>
+      <c r="E18" s="136"/>
+      <c r="F18" s="136"/>
+      <c r="G18" s="136"/>
+      <c r="H18" s="136"/>
+      <c r="I18" s="136"/>
+      <c r="J18" s="136"/>
+      <c r="K18" s="136"/>
+      <c r="L18" s="137"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -14622,10 +14202,10 @@
       <c r="B4" s="41"/>
     </row>
     <row r="6" spans="1:12" ht="18" x14ac:dyDescent="0.35">
-      <c r="A6" s="152" t="s">
+      <c r="A6" s="66" t="s">
         <v>44</v>
       </c>
-      <c r="B6" s="152"/>
+      <c r="B6" s="66"/>
     </row>
     <row r="8" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="44" t="s">
@@ -15230,12 +14810,56 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="8029d101-3d2a-47c4-b15f-619642bf5e50">
+      <UserInfo>
+        <DisplayName>Luis Campos / Logiztik Alliance</DisplayName>
+        <AccountId>265</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Jairo Gonzalez / Logiztik Alliance</DisplayName>
+        <AccountId>322</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>José Ganchozo / Logiztik Alliance</DisplayName>
+        <AccountId>304</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Edwin Casa / Logiztik Alliance</DisplayName>
+        <AccountId>299</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Cristhian Cuichan / Logiztik Alliance</DisplayName>
+        <AccountId>369</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Oscar Yunda /  Logiztik Alliance</DisplayName>
+        <AccountId>355</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Fernando Ordoñez / Logiztik Alliance</DisplayName>
+        <AccountId>321</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Alex Rivera / Logiztik Alliance</DisplayName>
+        <AccountId>370</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <TaxCatchAll xmlns="8029d101-3d2a-47c4-b15f-619642bf5e50" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87481c51-c14c-4071-bf64-faa2b5708bb6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -15488,62 +15112,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="8029d101-3d2a-47c4-b15f-619642bf5e50">
-      <UserInfo>
-        <DisplayName>Luis Campos / Logiztik Alliance</DisplayName>
-        <AccountId>265</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Jairo Gonzalez / Logiztik Alliance</DisplayName>
-        <AccountId>322</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>José Ganchozo / Logiztik Alliance</DisplayName>
-        <AccountId>304</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Edwin Casa / Logiztik Alliance</DisplayName>
-        <AccountId>299</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Cristhian Cuichan / Logiztik Alliance</DisplayName>
-        <AccountId>369</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Oscar Yunda /  Logiztik Alliance</DisplayName>
-        <AccountId>355</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Fernando Ordoñez / Logiztik Alliance</DisplayName>
-        <AccountId>321</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Alex Rivera / Logiztik Alliance</DisplayName>
-        <AccountId>370</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <TaxCatchAll xmlns="8029d101-3d2a-47c4-b15f-619642bf5e50" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87481c51-c14c-4071-bf64-faa2b5708bb6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{371D8832-41B3-447B-B13D-2663C267E34F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD069904-634F-48DA-AA92-BAE250498BEE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="8029d101-3d2a-47c4-b15f-619642bf5e50"/>
+    <ds:schemaRef ds:uri="87481c51-c14c-4071-bf64-faa2b5708bb6"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -15568,12 +15151,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD069904-634F-48DA-AA92-BAE250498BEE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{371D8832-41B3-447B-B13D-2663C267E34F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="8029d101-3d2a-47c4-b15f-619642bf5e50"/>
-    <ds:schemaRef ds:uri="87481c51-c14c-4071-bf64-faa2b5708bb6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>